<commit_message>
Exclude display-only units from change events
</commit_message>
<xml_diff>
--- a/outputs/weekly_unit_change_database.xlsx
+++ b/outputs/weekly_unit_change_database.xlsx
@@ -17,9 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'房源变化'!$A$1:$N$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'房源变化'!$A$1:$N$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'降价房源'!$A$1:$N$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'新增房源'!$A$1:$N$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'新增房源'!$A$1:$N$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'售出房源'!$A$1:$N$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'其他变化'!$A$1:$N$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'当前房源数据库'!$A$1:$J$716</definedName>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N115"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
@@ -3938,35 +3938,39 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>SE3 - Kidbrooke Village</t>
+          <t>SW19 - Wimbledon Bridge House (London Square)</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2-3-4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
+          <t>1 Bed</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>29.06.26</t>
+          <t>15.06.26</t>
         </is>
       </c>
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>06.07.26</t>
+          <t>29.06.26</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3975,15 +3979,11 @@
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr"/>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>Show Apartment</t>
-        </is>
-      </c>
+      <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="n"/>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T16:53:11</t>
+          <t>2026-07-08T17:02:25</t>
         </is>
       </c>
     </row>
@@ -3995,22 +3995,22 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>102</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="F66" s="2" t="n"/>
@@ -4019,7 +4019,9 @@
           <t>15.06.26</t>
         </is>
       </c>
-      <c r="H66" s="2" t="n"/>
+      <c r="H66" s="3" t="n">
+        <v>1185000</v>
+      </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
           <t>29.06.26</t>
@@ -4047,7 +4049,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>104</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -4057,12 +4059,12 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>West</t>
         </is>
       </c>
       <c r="F67" s="2" t="n"/>
@@ -4072,7 +4074,7 @@
         </is>
       </c>
       <c r="H67" s="3" t="n">
-        <v>1185000</v>
+        <v>710000</v>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
@@ -4101,22 +4103,22 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>Suite</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="F68" s="2" t="n"/>
@@ -4126,7 +4128,7 @@
         </is>
       </c>
       <c r="H68" s="3" t="n">
-        <v>710000</v>
+        <v>512500</v>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
@@ -4155,12 +4157,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>56</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -4180,7 +4182,7 @@
         </is>
       </c>
       <c r="H69" s="3" t="n">
-        <v>512500</v>
+        <v>507500</v>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
@@ -4209,12 +4211,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>71</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -4234,7 +4236,7 @@
         </is>
       </c>
       <c r="H70" s="3" t="n">
-        <v>507500</v>
+        <v>517500</v>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
@@ -4263,22 +4265,22 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>93</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Suite</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="F71" s="2" t="n"/>
@@ -4288,7 +4290,7 @@
         </is>
       </c>
       <c r="H71" s="3" t="n">
-        <v>517500</v>
+        <v>720000</v>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
@@ -4317,17 +4319,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -4335,15 +4337,15 @@
           <t>North</t>
         </is>
       </c>
-      <c r="F72" s="2" t="n"/>
+      <c r="F72" s="3" t="n">
+        <v>1225000</v>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
           <t>15.06.26</t>
         </is>
       </c>
-      <c r="H72" s="3" t="n">
-        <v>720000</v>
-      </c>
+      <c r="H72" s="2" t="n"/>
       <c r="I72" s="2" t="inlineStr">
         <is>
           <t>29.06.26</t>
@@ -4351,11 +4353,15 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>NEW_RELEASE</t>
+          <t>SOLD</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>缺失</t>
+        </is>
+      </c>
       <c r="M72" s="2" t="n"/>
       <c r="N72" s="2" t="inlineStr">
         <is>
@@ -4371,26 +4377,26 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>27</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>Suite</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>1225000</v>
+        <v>502500</v>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
@@ -4429,12 +4435,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>64</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -4444,11 +4450,11 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="F74" s="3" t="n">
-        <v>502500</v>
+        <v>512500</v>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
@@ -4487,7 +4493,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -4497,17 +4503,15 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Suite</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>North</t>
-        </is>
-      </c>
-      <c r="F75" s="3" t="n">
-        <v>512500</v>
-      </c>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
           <t>15.06.26</t>
@@ -4545,12 +4549,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -4560,10 +4564,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="n"/>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>597500</v>
+      </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
           <t>15.06.26</t>
@@ -4601,26 +4607,26 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>Suite</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>597500</v>
+        <v>517500</v>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
@@ -4659,26 +4665,26 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Suite</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>South East</t>
         </is>
       </c>
       <c r="F78" s="3" t="n">
-        <v>517500</v>
+        <v>740000</v>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
@@ -4712,58 +4718,50 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>SW19 - Wimbledon Bridge House (London Square)</t>
+          <t>SW6 - Chelsea Waterfront Tower East</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>30.2</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>South East</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="n">
-        <v>740000</v>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>15.06.26</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="n"/>
+          <t>8th June 2026</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="n">
+        <v>5842000</v>
+      </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>29.06.26</t>
+          <t>29th June 2026</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>SOLD</t>
+          <t>NEW_RELEASE</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
-      <c r="L79" s="2" t="inlineStr">
-        <is>
-          <t>缺失</t>
-        </is>
-      </c>
+      <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="n"/>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T17:02:25</t>
+          <t>2026-07-08T17:02:57</t>
         </is>
       </c>
     </row>
@@ -4775,12 +4773,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -4795,9 +4793,7 @@
           <t>8th June 2026</t>
         </is>
       </c>
-      <c r="H80" s="3" t="n">
-        <v>5842000</v>
-      </c>
+      <c r="H80" s="2" t="n"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
           <t>29th June 2026</t>
@@ -4805,11 +4801,15 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>NEW_RELEASE</t>
+          <t>SOLD</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
-      <c r="L80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>缺失</t>
+        </is>
+      </c>
       <c r="M80" s="2" t="n"/>
       <c r="N80" s="2" t="inlineStr">
         <is>
@@ -4820,52 +4820,54 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>SW6 - Chelsea Waterfront Tower East</t>
+          <t>SW6 - King's Road Park</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>G1.3-01-04</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr"/>
+          <t>2 Bedroom</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>S/W - Park Views</t>
+        </is>
+      </c>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>8th June 2026</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="n"/>
+          <t>28.06.2026</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="n">
+        <v>1370000</v>
+      </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>29th June 2026</t>
+          <t>05.07.2026</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>SOLD</t>
+          <t>NEW_RELEASE</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr"/>
-      <c r="L81" s="2" t="inlineStr">
-        <is>
-          <t>缺失</t>
-        </is>
-      </c>
+      <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="n"/>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T17:02:57</t>
+          <t>2026-07-08T16:53:34</t>
         </is>
       </c>
     </row>
@@ -4877,12 +4879,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>G1.3-01-04</t>
+          <t>G1.4-00-06</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4892,7 +4894,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>S/W - Park Views</t>
+          <t>S – Park Views</t>
         </is>
       </c>
       <c r="F82" s="2" t="n"/>
@@ -4901,9 +4903,7 @@
           <t>28.06.2026</t>
         </is>
       </c>
-      <c r="H82" s="3" t="n">
-        <v>1370000</v>
-      </c>
+      <c r="H82" s="2" t="n"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
           <t>05.07.2026</t>
@@ -4931,31 +4931,35 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>G1.4-00-06</t>
+          <t>H1-19-06</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>2 Bedroom</t>
+          <t>3 Bedroom</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>S – Park Views</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="n"/>
+          <t>South / West</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>2975500</v>
+      </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
           <t>28.06.2026</t>
         </is>
       </c>
-      <c r="H83" s="2" t="n"/>
+      <c r="H83" s="3" t="n">
+        <v>2975000</v>
+      </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
           <t>05.07.2026</t>
@@ -4963,73 +4967,71 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>NEW_RELEASE</t>
+          <t>PRICE_DROP</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
-      <c r="M83" s="2" t="n"/>
+      <c r="M83" s="2" t="n">
+        <v>-500</v>
+      </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T16:53:34</t>
+          <t>2026-07-08T16:53:41</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>SW6 - King's Road Park</t>
+          <t>UB1 - The Green Quarter</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>H1-19-06</t>
+          <t>257</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>3 Bedroom</t>
+          <t>2 Bed 2 Bath</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>South / West</t>
-        </is>
-      </c>
-      <c r="F84" s="3" t="n">
-        <v>2975500</v>
-      </c>
+          <t>S &amp; E</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>28.06.2026</t>
+          <t>28.06.26</t>
         </is>
       </c>
       <c r="H84" s="3" t="n">
-        <v>2975000</v>
+        <v>545000</v>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>05.07.2026</t>
+          <t>05.07.26</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>PRICE_DROP</t>
+          <t>NEW_RELEASE</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
-      <c r="M84" s="2" t="n">
-        <v>-500</v>
-      </c>
+      <c r="M84" s="2" t="n"/>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T16:53:41</t>
+          <t>2026-07-09T11:09:36</t>
         </is>
       </c>
     </row>
@@ -5041,22 +5043,22 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>261</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>2 Bed 2 Bath</t>
+          <t>2 Bed 2.5 Bath</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>S &amp; E</t>
+          <t>N &amp; W</t>
         </is>
       </c>
       <c r="F85" s="2" t="n"/>
@@ -5066,7 +5068,7 @@
         </is>
       </c>
       <c r="H85" s="3" t="n">
-        <v>545000</v>
+        <v>555000</v>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
@@ -5095,12 +5097,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>261</t>
+          <t>269</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -5120,7 +5122,7 @@
         </is>
       </c>
       <c r="H86" s="3" t="n">
-        <v>555000</v>
+        <v>565000</v>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
@@ -5149,12 +5151,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>285</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -5174,7 +5176,7 @@
         </is>
       </c>
       <c r="H87" s="3" t="n">
-        <v>565000</v>
+        <v>575000</v>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
@@ -5203,33 +5205,33 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>300</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>2 Bed 2.5 Bath</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>N &amp; W</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="n"/>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>400000</v>
+      </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H88" s="3" t="n">
-        <v>575000</v>
-      </c>
+      <c r="H88" s="2" t="n"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -5237,11 +5239,15 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>NEW_RELEASE</t>
+          <t>RESERVED</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>ON HOLD</t>
+        </is>
+      </c>
       <c r="M88" s="2" t="n"/>
       <c r="N88" s="2" t="inlineStr">
         <is>
@@ -5257,17 +5263,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>291</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -5275,9 +5281,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="F89" s="3" t="n">
-        <v>400000</v>
-      </c>
+      <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -5291,13 +5295,17 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
+          <t>SOLD</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
           <t>RESERVED</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr"/>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>ON HOLD</t>
+          <t>缺失</t>
         </is>
       </c>
       <c r="M89" s="2" t="n"/>
@@ -5315,17 +5323,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>308</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -5370,60 +5378,58 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>UB1 - The Green Quarter</t>
+          <t>W12 - White City Living</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>V18.02</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>3+Study</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="n"/>
+          <t>South/West/North</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>2850000</v>
+      </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>28.06.26</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="n"/>
+          <t>27.06.26</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="n">
+        <v>2815000</v>
+      </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>05.07.26</t>
+          <t>02.07.26</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>SOLD</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr">
-        <is>
-          <t>RESERVED</t>
-        </is>
-      </c>
-      <c r="L91" s="2" t="inlineStr">
-        <is>
-          <t>缺失</t>
-        </is>
-      </c>
-      <c r="M91" s="2" t="n"/>
+          <t>PRICE_DROP</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="n">
+        <v>-35000</v>
+      </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T11:09:36</t>
+          <t>2026-07-09T09:53:11</t>
         </is>
       </c>
     </row>
@@ -5435,34 +5441,32 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>V18.02</t>
+          <t>W.14.03</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>3+Study</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>South/West/North</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="n">
-        <v>2850000</v>
-      </c>
+          <t>North/East</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
           <t>27.06.26</t>
         </is>
       </c>
       <c r="H92" s="3" t="n">
-        <v>2815000</v>
+        <v>775000</v>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
@@ -5471,17 +5475,15 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>PRICE_DROP</t>
+          <t>NEW_RELEASE</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr"/>
-      <c r="M92" s="2" t="n">
-        <v>-35000</v>
-      </c>
+      <c r="M92" s="2" t="n"/>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T09:53:11</t>
+          <t>2026-07-08T17:01:26</t>
         </is>
       </c>
     </row>
@@ -5493,32 +5495,34 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>W.14.03</t>
+          <t>W.30.01</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>30/31</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Penthouse</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>North/East</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="n"/>
+          <t>South/West/North</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>4000000</v>
+      </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
           <t>27.06.26</t>
         </is>
       </c>
       <c r="H93" s="3" t="n">
-        <v>775000</v>
+        <v>3990000</v>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
@@ -5527,12 +5531,14 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>NEW_RELEASE</t>
+          <t>PRICE_DROP</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr"/>
-      <c r="M93" s="2" t="n"/>
+      <c r="M93" s="2" t="n">
+        <v>-10000</v>
+      </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
           <t>2026-07-08T17:01:26</t>
@@ -5547,7 +5553,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>W.30.01</t>
+          <t>W.30.02</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -5562,7 +5568,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>South/West/North</t>
+          <t>South/East/North</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -5605,35 +5611,33 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>W.30.02</t>
+          <t>W.08.01</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>30/31</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Penthouse</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>South/East/North</t>
+          <t>North/West</t>
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>4000000</v>
+        <v>775000</v>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
           <t>27.06.26</t>
         </is>
       </c>
-      <c r="H95" s="3" t="n">
-        <v>3990000</v>
-      </c>
+      <c r="H95" s="2" t="n"/>
       <c r="I95" s="2" t="inlineStr">
         <is>
           <t>02.07.26</t>
@@ -5641,14 +5645,16 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>PRICE_DROP</t>
+          <t>SOLD</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr"/>
-      <c r="M95" s="2" t="n">
-        <v>-10000</v>
-      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>缺失</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="n"/>
       <c r="N95" s="2" t="inlineStr">
         <is>
           <t>2026-07-08T17:01:26</t>
@@ -5663,12 +5669,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>W.08.01</t>
+          <t>W.14.01</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -5681,9 +5687,7 @@
           <t>North/West</t>
         </is>
       </c>
-      <c r="F96" s="3" t="n">
-        <v>775000</v>
-      </c>
+      <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
           <t>27.06.26</t>
@@ -5716,22 +5720,22 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>W12 - White City Living</t>
+          <t>W2 - Trillium</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>W.14.01</t>
+          <t>I.01.07</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -5742,30 +5746,26 @@
       <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>27.06.26</t>
+          <t>28.06.26</t>
         </is>
       </c>
       <c r="H97" s="2" t="n"/>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>02.07.26</t>
+          <t>05.07.26</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>SOLD</t>
+          <t>NEW_RELEASE</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
-      <c r="L97" s="2" t="inlineStr">
-        <is>
-          <t>缺失</t>
-        </is>
-      </c>
+      <c r="L97" s="2" t="inlineStr"/>
       <c r="M97" s="2" t="n"/>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T17:01:26</t>
+          <t>2026-07-08T16:56:04</t>
         </is>
       </c>
     </row>
@@ -5777,22 +5777,22 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>I.01.07</t>
+          <t>I.08.05</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
+          <t>South/West</t>
         </is>
       </c>
       <c r="F98" s="2" t="n"/>
@@ -5829,22 +5829,22 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>I.08.05</t>
+          <t>I.10.07</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>South/West</t>
+          <t>North/West</t>
         </is>
       </c>
       <c r="F99" s="2" t="n"/>
@@ -5881,22 +5881,22 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>I.10.07</t>
+          <t>I.14.01</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
+          <t>North/East</t>
         </is>
       </c>
       <c r="F100" s="2" t="n"/>
@@ -5905,7 +5905,9 @@
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H100" s="2" t="n"/>
+      <c r="H100" s="3" t="n">
+        <v>1598500</v>
+      </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -5933,7 +5935,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>I.14.01</t>
+          <t>I.14.06</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -5943,12 +5945,12 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>North/East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="F101" s="2" t="n"/>
@@ -5957,9 +5959,7 @@
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H101" s="3" t="n">
-        <v>1598500</v>
-      </c>
+      <c r="H101" s="2" t="n"/>
       <c r="I101" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -5987,22 +5987,22 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>I.14.06</t>
+          <t>I.17.03</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>I</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="F102" s="2" t="n"/>
@@ -6039,22 +6039,22 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>I.17.03</t>
+          <t>I.20.06</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>North/West</t>
         </is>
       </c>
       <c r="F103" s="2" t="n"/>
@@ -6063,7 +6063,9 @@
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H103" s="2" t="n"/>
+      <c r="H103" s="3" t="n">
+        <v>2505000</v>
+      </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -6091,33 +6093,33 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>I.20.06</t>
+          <t>I.02.05</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="n"/>
+          <t>South/ West</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>1350000</v>
+      </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H104" s="3" t="n">
-        <v>2505000</v>
-      </c>
+      <c r="H104" s="2" t="n"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -6125,11 +6127,15 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>NEW_RELEASE</t>
+          <t>SOLD</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr"/>
-      <c r="L104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>缺失</t>
+        </is>
+      </c>
       <c r="M104" s="2" t="n"/>
       <c r="N104" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6151,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>I.02.05</t>
+          <t>I.02.07</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -6155,17 +6161,15 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>South/ West</t>
-        </is>
-      </c>
-      <c r="F105" s="3" t="n">
-        <v>1350000</v>
-      </c>
+          <t>North/West</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -6203,12 +6207,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>I.02.07</t>
+          <t>I.07.07</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -6221,7 +6225,9 @@
           <t>North/West</t>
         </is>
       </c>
-      <c r="F106" s="2" t="n"/>
+      <c r="F106" s="3" t="n">
+        <v>2005000</v>
+      </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -6259,27 +6265,25 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>I.07.07</t>
+          <t>I.13.01</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="n">
-        <v>2005000</v>
-      </c>
+          <t>North/East</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -6317,7 +6321,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>I.13.01</t>
+          <t>I.13.07</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -6327,15 +6331,17 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>North/East</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="n"/>
+          <t>North/West</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>2181500</v>
+      </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -6373,26 +6379,26 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>I.13.07</t>
+          <t>I.15.03</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>I</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="F109" s="3" t="n">
-        <v>2181500</v>
+        <v>1199000</v>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
@@ -6431,7 +6437,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>I.15.03</t>
+          <t>I.15.05</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -6441,17 +6447,15 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="n">
-        <v>1199000</v>
-      </c>
+          <t>South/West</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -6489,25 +6493,27 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>I.15.05</t>
+          <t>I.17.04</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>J</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>South/West</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="n"/>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>1115000</v>
+      </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
           <t>28.06.26</t>
@@ -6545,26 +6551,26 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>I.17.04</t>
+          <t>I.20.01</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>North/East</t>
         </is>
       </c>
       <c r="F112" s="3" t="n">
-        <v>1115000</v>
+        <v>1845000</v>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
@@ -6603,12 +6609,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>I.20.01</t>
+          <t>I.22.01</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -6622,7 +6628,7 @@
         </is>
       </c>
       <c r="F113" s="3" t="n">
-        <v>1845000</v>
+        <v>1897000</v>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
@@ -6661,7 +6667,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>I.22.01</t>
+          <t>I.22.04*</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -6671,16 +6677,16 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>J</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>North/East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="F114" s="3" t="n">
-        <v>1897000</v>
+        <v>1205000</v>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
@@ -6711,66 +6717,8 @@
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>W2 - Trillium</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
-        <is>
-          <t>I.22.04*</t>
-        </is>
-      </c>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="n">
-        <v>1205000</v>
-      </c>
-      <c r="G115" s="2" t="inlineStr">
-        <is>
-          <t>28.06.26</t>
-        </is>
-      </c>
-      <c r="H115" s="2" t="n"/>
-      <c r="I115" s="2" t="inlineStr">
-        <is>
-          <t>05.07.26</t>
-        </is>
-      </c>
-      <c r="J115" s="2" t="inlineStr">
-        <is>
-          <t>SOLD</t>
-        </is>
-      </c>
-      <c r="K115" s="2" t="inlineStr"/>
-      <c r="L115" s="2" t="inlineStr">
-        <is>
-          <t>缺失</t>
-        </is>
-      </c>
-      <c r="M115" s="2" t="n"/>
-      <c r="N115" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08T16:56:04</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N115"/>
+  <autoFilter ref="A1:N114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7848,7 +7796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7862,7 +7810,7 @@
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
@@ -9636,35 +9584,39 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SE3 - Kidbrooke Village</t>
+          <t>SW19 - Wimbledon Bridge House (London Square)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2-3-4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
+          <t>1 Bed</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>29.06.26</t>
+          <t>15.06.26</t>
         </is>
       </c>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>06.07.26</t>
+          <t>29.06.26</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -9673,15 +9625,11 @@
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>Show Apartment</t>
-        </is>
-      </c>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T16:53:11</t>
+          <t>2026-07-08T17:02:25</t>
         </is>
       </c>
     </row>
@@ -9693,22 +9641,22 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>102</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>2 Bed</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
@@ -9717,7 +9665,9 @@
           <t>15.06.26</t>
         </is>
       </c>
-      <c r="H35" s="2" t="n"/>
+      <c r="H35" s="3" t="n">
+        <v>1185000</v>
+      </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>29.06.26</t>
@@ -9745,7 +9695,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>104</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -9755,12 +9705,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2 Bed</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>West</t>
         </is>
       </c>
       <c r="F36" s="2" t="n"/>
@@ -9770,7 +9720,7 @@
         </is>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1185000</v>
+        <v>710000</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
@@ -9799,22 +9749,22 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
+          <t>Suite</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="F37" s="2" t="n"/>
@@ -9824,7 +9774,7 @@
         </is>
       </c>
       <c r="H37" s="3" t="n">
-        <v>710000</v>
+        <v>512500</v>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
@@ -9853,12 +9803,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>56</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -9878,7 +9828,7 @@
         </is>
       </c>
       <c r="H38" s="3" t="n">
-        <v>512500</v>
+        <v>507500</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
@@ -9907,12 +9857,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>71</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -9932,7 +9882,7 @@
         </is>
       </c>
       <c r="H39" s="3" t="n">
-        <v>507500</v>
+        <v>517500</v>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
@@ -9961,22 +9911,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>93</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Suite</t>
+          <t>1 Bed</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="F40" s="2" t="n"/>
@@ -9986,7 +9936,7 @@
         </is>
       </c>
       <c r="H40" s="3" t="n">
-        <v>517500</v>
+        <v>720000</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
@@ -10010,41 +9960,37 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SW19 - Wimbledon Bridge House (London Square)</t>
+          <t>SW6 - Chelsea Waterfront Tower East</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>30.2</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1 Bed</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>North</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>15.06.26</t>
+          <t>8th June 2026</t>
         </is>
       </c>
       <c r="H41" s="3" t="n">
-        <v>720000</v>
+        <v>5842000</v>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>29.06.26</t>
+          <t>29th June 2026</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -10057,44 +10003,48 @@
       <c r="M41" s="2" t="n"/>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T17:02:25</t>
+          <t>2026-07-08T17:02:57</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SW6 - Chelsea Waterfront Tower East</t>
+          <t>SW6 - King's Road Park</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>G1.3-01-04</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
+          <t>2 Bedroom</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>S/W - Park Views</t>
+        </is>
+      </c>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>8th June 2026</t>
+          <t>28.06.2026</t>
         </is>
       </c>
       <c r="H42" s="3" t="n">
-        <v>5842000</v>
+        <v>1370000</v>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>29th June 2026</t>
+          <t>05.07.2026</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -10107,7 +10057,7 @@
       <c r="M42" s="2" t="n"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T17:02:57</t>
+          <t>2026-07-08T16:53:34</t>
         </is>
       </c>
     </row>
@@ -10119,12 +10069,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>G1.3-01-04</t>
+          <t>G1.4-00-06</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -10134,7 +10084,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>S/W - Park Views</t>
+          <t>S – Park Views</t>
         </is>
       </c>
       <c r="F43" s="2" t="n"/>
@@ -10143,9 +10093,7 @@
           <t>28.06.2026</t>
         </is>
       </c>
-      <c r="H43" s="3" t="n">
-        <v>1370000</v>
-      </c>
+      <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>05.07.2026</t>
@@ -10168,39 +10116,41 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>SW6 - King's Road Park</t>
+          <t>UB1 - The Green Quarter</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>G1.4-00-06</t>
+          <t>257</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2 Bedroom</t>
+          <t>2 Bed 2 Bath</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>S – Park Views</t>
+          <t>S &amp; E</t>
         </is>
       </c>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>28.06.2026</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="n"/>
+          <t>28.06.26</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>545000</v>
+      </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>05.07.2026</t>
+          <t>05.07.26</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -10213,7 +10163,7 @@
       <c r="M44" s="2" t="n"/>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T16:53:34</t>
+          <t>2026-07-09T11:09:36</t>
         </is>
       </c>
     </row>
@@ -10225,22 +10175,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>261</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2 Bed 2 Bath</t>
+          <t>2 Bed 2.5 Bath</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>S &amp; E</t>
+          <t>N &amp; W</t>
         </is>
       </c>
       <c r="F45" s="2" t="n"/>
@@ -10250,7 +10200,7 @@
         </is>
       </c>
       <c r="H45" s="3" t="n">
-        <v>545000</v>
+        <v>555000</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -10279,12 +10229,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>261</t>
+          <t>269</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -10304,7 +10254,7 @@
         </is>
       </c>
       <c r="H46" s="3" t="n">
-        <v>555000</v>
+        <v>565000</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
@@ -10333,12 +10283,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>285</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -10358,7 +10308,7 @@
         </is>
       </c>
       <c r="H47" s="3" t="n">
-        <v>565000</v>
+        <v>575000</v>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
@@ -10382,41 +10332,41 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>UB1 - The Green Quarter</t>
+          <t>W12 - White City Living</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>W.14.03</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2 Bed 2.5 Bath</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>N &amp; W</t>
+          <t>North/East</t>
         </is>
       </c>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>28.06.26</t>
+          <t>27.06.26</t>
         </is>
       </c>
       <c r="H48" s="3" t="n">
-        <v>575000</v>
+        <v>775000</v>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>05.07.26</t>
+          <t>02.07.26</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -10429,48 +10379,46 @@
       <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T11:09:36</t>
+          <t>2026-07-08T17:01:26</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>W12 - White City Living</t>
+          <t>W2 - Trillium</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>W.14.03</t>
+          <t>I.01.07</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>North/East</t>
+          <t>North/West</t>
         </is>
       </c>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>27.06.26</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="n">
-        <v>775000</v>
-      </c>
+          <t>28.06.26</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>02.07.26</t>
+          <t>05.07.26</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -10483,7 +10431,7 @@
       <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08T17:01:26</t>
+          <t>2026-07-08T16:56:04</t>
         </is>
       </c>
     </row>
@@ -10495,22 +10443,22 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>I.01.07</t>
+          <t>I.08.05</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
+          <t>South/West</t>
         </is>
       </c>
       <c r="F50" s="2" t="n"/>
@@ -10547,22 +10495,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>I.08.05</t>
+          <t>I.10.07</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>South/West</t>
+          <t>North/West</t>
         </is>
       </c>
       <c r="F51" s="2" t="n"/>
@@ -10599,22 +10547,22 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>I.10.07</t>
+          <t>I.14.01</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>North/West</t>
+          <t>North/East</t>
         </is>
       </c>
       <c r="F52" s="2" t="n"/>
@@ -10623,7 +10571,9 @@
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H52" s="2" t="n"/>
+      <c r="H52" s="3" t="n">
+        <v>1598500</v>
+      </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -10651,7 +10601,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>I.14.01</t>
+          <t>I.14.06</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -10661,12 +10611,12 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>North/East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="F53" s="2" t="n"/>
@@ -10675,9 +10625,7 @@
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H53" s="3" t="n">
-        <v>1598500</v>
-      </c>
+      <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -10705,22 +10653,22 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>I.14.06</t>
+          <t>I.17.03</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>I</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="F54" s="2" t="n"/>
@@ -10757,22 +10705,22 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>I.17.03</t>
+          <t>I.20.06</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>North/West</t>
         </is>
       </c>
       <c r="F55" s="2" t="n"/>
@@ -10781,7 +10729,9 @@
           <t>28.06.26</t>
         </is>
       </c>
-      <c r="H55" s="2" t="n"/>
+      <c r="H55" s="3" t="n">
+        <v>2505000</v>
+      </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
           <t>05.07.26</t>
@@ -10801,62 +10751,8 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>W2 - Trillium</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>I.20.06</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>North/West</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>28.06.26</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="n">
-        <v>2505000</v>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>05.07.26</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>NEW_RELEASE</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr"/>
-      <c r="M56" s="2" t="n"/>
-      <c r="N56" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-08T16:56:04</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N56"/>
+  <autoFilter ref="A1:N55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh pricelist scan outputs
</commit_message>
<xml_diff>
--- a/outputs/weekly_unit_change_database.xlsx
+++ b/outputs/weekly_unit_change_database.xlsx
@@ -58854,7 +58854,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -58917,11 +58917,7 @@
           <t>E14 - South Quay Plaza</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>E14 - South Quay Plaza · sqp</t>
-        </is>
-      </c>
+      <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>SQP Daily Price List 25.06.2026.pdf</t>
@@ -58932,17 +58928,11 @@
           <t>SQP Daily Price List 04.07.2026.pdf</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>